<commit_message>
Estadisticos Segundo Parcial 2624
</commit_message>
<xml_diff>
--- a/Calificaciones20232.xlsx
+++ b/Calificaciones20232.xlsx
@@ -3705,7 +3705,7 @@
         <v>5</v>
       </c>
       <c r="O4">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P4">
         <v>5</v>
@@ -3818,7 +3818,7 @@
         <v>9</v>
       </c>
       <c r="O5">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P5">
         <v>10</v>
@@ -3931,7 +3931,7 @@
         <v>8</v>
       </c>
       <c r="O6">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P6">
         <v>7</v>
@@ -4044,7 +4044,7 @@
         <v>10</v>
       </c>
       <c r="O7">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P7">
         <v>10</v>
@@ -4157,7 +4157,7 @@
         <v>6</v>
       </c>
       <c r="O8">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="P8">
         <v>7</v>
@@ -4270,7 +4270,7 @@
         <v>6</v>
       </c>
       <c r="O9">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="P9">
         <v>9</v>
@@ -4383,7 +4383,7 @@
         <v>8</v>
       </c>
       <c r="O10">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P10">
         <v>8</v>
@@ -4437,7 +4437,7 @@
         <v>9</v>
       </c>
       <c r="AG10">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AH10">
         <v>7</v>
@@ -4496,7 +4496,7 @@
         <v>9</v>
       </c>
       <c r="O11">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P11">
         <v>10</v>
@@ -4609,7 +4609,7 @@
         <v>9</v>
       </c>
       <c r="O12">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P12">
         <v>10</v>
@@ -4663,7 +4663,7 @@
         <v>10</v>
       </c>
       <c r="AG12">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AH12">
         <v>10</v>
@@ -4722,7 +4722,7 @@
         <v>9</v>
       </c>
       <c r="O13">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P13">
         <v>10</v>
@@ -4835,7 +4835,7 @@
         <v>7</v>
       </c>
       <c r="O14">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="P14">
         <v>10</v>
@@ -4948,7 +4948,7 @@
         <v>7</v>
       </c>
       <c r="O15">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="P15">
         <v>10</v>
@@ -5061,7 +5061,7 @@
         <v>5</v>
       </c>
       <c r="O16">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P16">
         <v>5</v>
@@ -5174,7 +5174,7 @@
         <v>5</v>
       </c>
       <c r="O17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P17">
         <v>5</v>
@@ -5228,7 +5228,7 @@
         <v>5</v>
       </c>
       <c r="AG17">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AH17">
         <v>5</v>
@@ -5287,7 +5287,7 @@
         <v>5</v>
       </c>
       <c r="O18">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P18">
         <v>5</v>
@@ -5400,7 +5400,7 @@
         <v>7</v>
       </c>
       <c r="O19">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P19">
         <v>5</v>
@@ -5513,7 +5513,7 @@
         <v>5</v>
       </c>
       <c r="O20">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="P20">
         <v>7</v>
@@ -5626,7 +5626,7 @@
         <v>6</v>
       </c>
       <c r="O21">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P21">
         <v>9</v>
@@ -5739,7 +5739,7 @@
         <v>6</v>
       </c>
       <c r="O22">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="P22">
         <v>7</v>
@@ -5852,7 +5852,7 @@
         <v>8</v>
       </c>
       <c r="O23">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P23">
         <v>10</v>
@@ -5965,7 +5965,7 @@
         <v>9</v>
       </c>
       <c r="O24">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P24">
         <v>10</v>
@@ -6019,7 +6019,7 @@
         <v>8</v>
       </c>
       <c r="AG24">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AH24">
         <v>9</v>
@@ -6078,7 +6078,7 @@
         <v>5</v>
       </c>
       <c r="O25">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P25">
         <v>5</v>
@@ -6191,7 +6191,7 @@
         <v>5</v>
       </c>
       <c r="O26">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="P26">
         <v>7</v>
@@ -6304,7 +6304,7 @@
         <v>8</v>
       </c>
       <c r="O27">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P27">
         <v>8</v>
@@ -6358,7 +6358,7 @@
         <v>9</v>
       </c>
       <c r="AG27">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AH27">
         <v>9</v>
@@ -6417,7 +6417,7 @@
         <v>5</v>
       </c>
       <c r="O28">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="P28">
         <v>5</v>
@@ -24106,7 +24106,7 @@
         <v>9</v>
       </c>
       <c r="H4">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I4">
         <v>10</v>
@@ -24183,7 +24183,7 @@
         <v>10</v>
       </c>
       <c r="H5">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I5">
         <v>10</v>
@@ -24219,7 +24219,7 @@
         <v>-1</v>
       </c>
       <c r="T5">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U5">
         <v>10</v>
@@ -24260,7 +24260,7 @@
         <v>10</v>
       </c>
       <c r="H6">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I6">
         <v>10</v>
@@ -24337,7 +24337,7 @@
         <v>9</v>
       </c>
       <c r="H7">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I7">
         <v>8</v>
@@ -24373,7 +24373,7 @@
         <v>-1</v>
       </c>
       <c r="T7">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U7">
         <v>9</v>
@@ -24414,7 +24414,7 @@
         <v>9</v>
       </c>
       <c r="H8">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I8">
         <v>9</v>
@@ -24450,7 +24450,7 @@
         <v>-1</v>
       </c>
       <c r="T8">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U8">
         <v>9</v>
@@ -24491,7 +24491,7 @@
         <v>6</v>
       </c>
       <c r="H9">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I9">
         <v>8</v>
@@ -24527,7 +24527,7 @@
         <v>-1</v>
       </c>
       <c r="T9">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U9">
         <v>9</v>
@@ -24568,7 +24568,7 @@
         <v>10</v>
       </c>
       <c r="H10">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I10">
         <v>8</v>
@@ -24604,7 +24604,7 @@
         <v>-1</v>
       </c>
       <c r="T10">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U10">
         <v>9</v>
@@ -24645,7 +24645,7 @@
         <v>8</v>
       </c>
       <c r="H11">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I11">
         <v>10</v>
@@ -24722,7 +24722,7 @@
         <v>8</v>
       </c>
       <c r="H12">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I12">
         <v>10</v>
@@ -24758,7 +24758,7 @@
         <v>-1</v>
       </c>
       <c r="T12">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U12">
         <v>10</v>
@@ -24799,7 +24799,7 @@
         <v>9</v>
       </c>
       <c r="H13">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I13">
         <v>10</v>
@@ -24835,7 +24835,7 @@
         <v>-1</v>
       </c>
       <c r="T13">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U13">
         <v>10</v>
@@ -24876,7 +24876,7 @@
         <v>8</v>
       </c>
       <c r="H14">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I14">
         <v>10</v>
@@ -24912,7 +24912,7 @@
         <v>-1</v>
       </c>
       <c r="T14">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U14">
         <v>10</v>
@@ -24953,7 +24953,7 @@
         <v>10</v>
       </c>
       <c r="H15">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I15">
         <v>10</v>
@@ -25030,7 +25030,7 @@
         <v>7</v>
       </c>
       <c r="H16">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I16">
         <v>9</v>
@@ -25066,7 +25066,7 @@
         <v>-1</v>
       </c>
       <c r="T16">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U16">
         <v>9</v>
@@ -25107,7 +25107,7 @@
         <v>6</v>
       </c>
       <c r="H17">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I17">
         <v>8</v>
@@ -25143,7 +25143,7 @@
         <v>-1</v>
       </c>
       <c r="T17">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U17">
         <v>8</v>
@@ -25184,7 +25184,7 @@
         <v>10</v>
       </c>
       <c r="H18">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I18">
         <v>10</v>
@@ -25261,7 +25261,7 @@
         <v>9</v>
       </c>
       <c r="H19">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I19">
         <v>10</v>
@@ -25338,7 +25338,7 @@
         <v>10</v>
       </c>
       <c r="H20">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I20">
         <v>10</v>
@@ -25415,7 +25415,7 @@
         <v>9</v>
       </c>
       <c r="H21">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I21">
         <v>9</v>
@@ -25492,7 +25492,7 @@
         <v>8</v>
       </c>
       <c r="H22">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I22">
         <v>8</v>
@@ -25528,7 +25528,7 @@
         <v>-1</v>
       </c>
       <c r="T22">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U22">
         <v>8</v>
@@ -25569,7 +25569,7 @@
         <v>9</v>
       </c>
       <c r="H23">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I23">
         <v>9</v>
@@ -25605,7 +25605,7 @@
         <v>-1</v>
       </c>
       <c r="T23">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U23">
         <v>9</v>
@@ -25646,7 +25646,7 @@
         <v>7</v>
       </c>
       <c r="H24">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I24">
         <v>10</v>
@@ -25682,7 +25682,7 @@
         <v>-1</v>
       </c>
       <c r="T24">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U24">
         <v>9</v>
@@ -25723,7 +25723,7 @@
         <v>9</v>
       </c>
       <c r="H25">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I25">
         <v>10</v>
@@ -25759,7 +25759,7 @@
         <v>-1</v>
       </c>
       <c r="T25">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U25">
         <v>9</v>
@@ -25800,7 +25800,7 @@
         <v>10</v>
       </c>
       <c r="H26">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I26">
         <v>10</v>
@@ -25877,7 +25877,7 @@
         <v>4</v>
       </c>
       <c r="H27">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I27">
         <v>10</v>
@@ -25913,7 +25913,7 @@
         <v>-1</v>
       </c>
       <c r="T27">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U27">
         <v>10</v>
@@ -25954,7 +25954,7 @@
         <v>9</v>
       </c>
       <c r="H28">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I28">
         <v>10</v>
@@ -26031,7 +26031,7 @@
         <v>7</v>
       </c>
       <c r="H29">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I29">
         <v>10</v>
@@ -26067,7 +26067,7 @@
         <v>-1</v>
       </c>
       <c r="T29">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U29">
         <v>9</v>
@@ -26108,7 +26108,7 @@
         <v>10</v>
       </c>
       <c r="H30">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I30">
         <v>8</v>
@@ -26144,7 +26144,7 @@
         <v>-1</v>
       </c>
       <c r="T30">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U30">
         <v>9</v>
@@ -26185,7 +26185,7 @@
         <v>9</v>
       </c>
       <c r="H31">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I31">
         <v>10</v>
@@ -26221,7 +26221,7 @@
         <v>-1</v>
       </c>
       <c r="T31">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U31">
         <v>10</v>
@@ -26262,7 +26262,7 @@
         <v>10</v>
       </c>
       <c r="H32">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I32">
         <v>10</v>
@@ -26339,7 +26339,7 @@
         <v>7</v>
       </c>
       <c r="H33">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I33">
         <v>8</v>
@@ -26375,7 +26375,7 @@
         <v>-1</v>
       </c>
       <c r="T33">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U33">
         <v>8</v>
@@ -26416,7 +26416,7 @@
         <v>6</v>
       </c>
       <c r="H34">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I34">
         <v>10</v>
@@ -26452,7 +26452,7 @@
         <v>-1</v>
       </c>
       <c r="T34">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U34">
         <v>9</v>
@@ -35546,7 +35546,7 @@
         <v>10</v>
       </c>
       <c r="N4">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O4">
         <v>7</v>
@@ -35659,7 +35659,7 @@
         <v>9</v>
       </c>
       <c r="N5">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="O5">
         <v>10</v>
@@ -35772,7 +35772,7 @@
         <v>8</v>
       </c>
       <c r="N6">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O6">
         <v>10</v>
@@ -35826,7 +35826,7 @@
         <v>8</v>
       </c>
       <c r="AF6">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AG6">
         <v>9</v>
@@ -35885,7 +35885,7 @@
         <v>6</v>
       </c>
       <c r="N7">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="O7">
         <v>9</v>
@@ -35998,7 +35998,7 @@
         <v>6</v>
       </c>
       <c r="N8">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="O8">
         <v>5</v>
@@ -36111,7 +36111,7 @@
         <v>8</v>
       </c>
       <c r="N9">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="O9">
         <v>8</v>
@@ -36224,7 +36224,7 @@
         <v>8</v>
       </c>
       <c r="N10">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O10">
         <v>10</v>
@@ -36278,7 +36278,7 @@
         <v>8</v>
       </c>
       <c r="AF10">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AG10">
         <v>10</v>
@@ -36337,7 +36337,7 @@
         <v>8</v>
       </c>
       <c r="N11">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O11">
         <v>8</v>
@@ -36391,7 +36391,7 @@
         <v>9</v>
       </c>
       <c r="AF11">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AG11">
         <v>9</v>
@@ -36450,7 +36450,7 @@
         <v>8</v>
       </c>
       <c r="N12">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O12">
         <v>10</v>
@@ -36563,7 +36563,7 @@
         <v>8</v>
       </c>
       <c r="N13">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O13">
         <v>10</v>
@@ -36676,7 +36676,7 @@
         <v>9</v>
       </c>
       <c r="N14">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O14">
         <v>10</v>
@@ -36730,7 +36730,7 @@
         <v>9</v>
       </c>
       <c r="AF14">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AG14">
         <v>9</v>
@@ -36789,7 +36789,7 @@
         <v>5</v>
       </c>
       <c r="N15">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="O15">
         <v>5</v>
@@ -36902,7 +36902,7 @@
         <v>8</v>
       </c>
       <c r="N16">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="O16">
         <v>10</v>
@@ -37015,7 +37015,7 @@
         <v>5</v>
       </c>
       <c r="N17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="O17">
         <v>5</v>
@@ -37128,7 +37128,7 @@
         <v>8</v>
       </c>
       <c r="N18">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="O18">
         <v>9</v>
@@ -37182,7 +37182,7 @@
         <v>8</v>
       </c>
       <c r="AF18">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AG18">
         <v>10</v>
@@ -37241,7 +37241,7 @@
         <v>8</v>
       </c>
       <c r="N19">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O19">
         <v>8</v>
@@ -37354,7 +37354,7 @@
         <v>7</v>
       </c>
       <c r="N20">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O20">
         <v>7</v>
@@ -37408,7 +37408,7 @@
         <v>6</v>
       </c>
       <c r="AF20">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AG20">
         <v>8</v>
@@ -37467,7 +37467,7 @@
         <v>5</v>
       </c>
       <c r="N21">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="O21">
         <v>5</v>
@@ -37580,7 +37580,7 @@
         <v>8</v>
       </c>
       <c r="N22">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O22">
         <v>7</v>
@@ -37693,7 +37693,7 @@
         <v>5</v>
       </c>
       <c r="N23">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="O23">
         <v>7</v>
@@ -37747,7 +37747,7 @@
         <v>5</v>
       </c>
       <c r="AF23">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AG23">
         <v>8</v>
@@ -37806,7 +37806,7 @@
         <v>6</v>
       </c>
       <c r="N24">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="O24">
         <v>8</v>
@@ -37919,7 +37919,7 @@
         <v>8</v>
       </c>
       <c r="N25">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O25">
         <v>9</v>
@@ -38032,7 +38032,7 @@
         <v>7</v>
       </c>
       <c r="N26">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O26">
         <v>8</v>
@@ -38145,7 +38145,7 @@
         <v>6</v>
       </c>
       <c r="N27">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="O27">
         <v>5</v>
@@ -38199,7 +38199,7 @@
         <v>7</v>
       </c>
       <c r="AF27">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AG27">
         <v>7</v>
@@ -38258,7 +38258,7 @@
         <v>7</v>
       </c>
       <c r="N28">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O28">
         <v>10</v>
@@ -38312,7 +38312,7 @@
         <v>8</v>
       </c>
       <c r="AF28">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AG28">
         <v>9</v>
@@ -38371,7 +38371,7 @@
         <v>8</v>
       </c>
       <c r="N29">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O29">
         <v>7</v>
@@ -38425,7 +38425,7 @@
         <v>9</v>
       </c>
       <c r="AF29">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AG29">
         <v>9</v>
@@ -38484,7 +38484,7 @@
         <v>9</v>
       </c>
       <c r="N30">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="O30">
         <v>9</v>
@@ -38597,7 +38597,7 @@
         <v>8</v>
       </c>
       <c r="N31">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O31">
         <v>10</v>
@@ -38710,7 +38710,7 @@
         <v>6</v>
       </c>
       <c r="N32">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="O32">
         <v>5</v>
@@ -38823,7 +38823,7 @@
         <v>8</v>
       </c>
       <c r="N33">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O33">
         <v>8</v>
@@ -38877,7 +38877,7 @@
         <v>8</v>
       </c>
       <c r="AF33">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AG33">
         <v>9</v>
@@ -38936,7 +38936,7 @@
         <v>10</v>
       </c>
       <c r="N34">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="O34">
         <v>10</v>
@@ -39049,7 +39049,7 @@
         <v>8</v>
       </c>
       <c r="N35">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O35">
         <v>8</v>
@@ -39103,7 +39103,7 @@
         <v>8</v>
       </c>
       <c r="AF35">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AG35">
         <v>9</v>
@@ -39162,7 +39162,7 @@
         <v>10</v>
       </c>
       <c r="N36">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="O36">
         <v>10</v>
@@ -39275,7 +39275,7 @@
         <v>8</v>
       </c>
       <c r="N37">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O37">
         <v>9</v>
@@ -39329,7 +39329,7 @@
         <v>9</v>
       </c>
       <c r="AF37">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AG37">
         <v>10</v>
@@ -39388,7 +39388,7 @@
         <v>7</v>
       </c>
       <c r="N38">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O38">
         <v>10</v>
@@ -39501,7 +39501,7 @@
         <v>6</v>
       </c>
       <c r="N39">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O39">
         <v>5</v>
@@ -39614,7 +39614,7 @@
         <v>7</v>
       </c>
       <c r="N40">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="O40">
         <v>5</v>
@@ -39727,7 +39727,7 @@
         <v>7</v>
       </c>
       <c r="N41">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O41">
         <v>10</v>
@@ -39840,7 +39840,7 @@
         <v>6</v>
       </c>
       <c r="N42">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="O42">
         <v>5</v>
@@ -77117,7 +77117,7 @@
         <v>117</v>
       </c>
       <c r="B4">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="C4">
         <v>8</v>
@@ -77144,7 +77144,7 @@
         <v>10</v>
       </c>
       <c r="K4">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="L4">
         <v>9</v>
@@ -77159,7 +77159,7 @@
         <v>10</v>
       </c>
       <c r="P4">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q4">
         <v>10</v>
@@ -77198,7 +77198,7 @@
         <v>-1</v>
       </c>
       <c r="AC4">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AD4">
         <v>9</v>
@@ -77230,7 +77230,7 @@
         <v>118</v>
       </c>
       <c r="B5">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="C5">
         <v>5</v>
@@ -77257,7 +77257,7 @@
         <v>10</v>
       </c>
       <c r="K5">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L5">
         <v>6</v>
@@ -77272,7 +77272,7 @@
         <v>7</v>
       </c>
       <c r="P5">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q5">
         <v>9</v>
@@ -77311,7 +77311,7 @@
         <v>-1</v>
       </c>
       <c r="AC5">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="AD5">
         <v>5</v>
@@ -77326,7 +77326,7 @@
         <v>8</v>
       </c>
       <c r="AH5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AI5">
         <v>8</v>
@@ -77343,7 +77343,7 @@
         <v>119</v>
       </c>
       <c r="B6">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="C6">
         <v>6</v>
@@ -77370,7 +77370,7 @@
         <v>10</v>
       </c>
       <c r="K6">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L6">
         <v>7</v>
@@ -77385,7 +77385,7 @@
         <v>9</v>
       </c>
       <c r="P6">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q6">
         <v>10</v>
@@ -77424,7 +77424,7 @@
         <v>-1</v>
       </c>
       <c r="AC6">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="AD6">
         <v>7</v>
@@ -77456,7 +77456,7 @@
         <v>120</v>
       </c>
       <c r="B7">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="C7">
         <v>5</v>
@@ -77483,7 +77483,7 @@
         <v>5</v>
       </c>
       <c r="K7">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L7">
         <v>5</v>
@@ -77498,7 +77498,7 @@
         <v>5</v>
       </c>
       <c r="P7">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q7">
         <v>5</v>
@@ -77537,7 +77537,7 @@
         <v>-1</v>
       </c>
       <c r="AC7">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="AD7">
         <v>5</v>
@@ -77569,7 +77569,7 @@
         <v>121</v>
       </c>
       <c r="B8">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="C8">
         <v>5</v>
@@ -77596,7 +77596,7 @@
         <v>5</v>
       </c>
       <c r="K8">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L8">
         <v>5</v>
@@ -77611,7 +77611,7 @@
         <v>5</v>
       </c>
       <c r="P8">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q8">
         <v>5</v>
@@ -77650,7 +77650,7 @@
         <v>-1</v>
       </c>
       <c r="AC8">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="AD8">
         <v>5</v>
@@ -77665,7 +77665,7 @@
         <v>6</v>
       </c>
       <c r="AH8">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AI8">
         <v>5</v>
@@ -77682,7 +77682,7 @@
         <v>122</v>
       </c>
       <c r="B9">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="C9">
         <v>5</v>
@@ -77709,7 +77709,7 @@
         <v>10</v>
       </c>
       <c r="K9">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="L9">
         <v>7</v>
@@ -77724,7 +77724,7 @@
         <v>9</v>
       </c>
       <c r="P9">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q9">
         <v>8</v>
@@ -77763,7 +77763,7 @@
         <v>-1</v>
       </c>
       <c r="AC9">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="AD9">
         <v>6</v>
@@ -77778,7 +77778,7 @@
         <v>7</v>
       </c>
       <c r="AH9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AI9">
         <v>7</v>
@@ -77795,7 +77795,7 @@
         <v>123</v>
       </c>
       <c r="B10">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="C10">
         <v>9</v>
@@ -77822,7 +77822,7 @@
         <v>10</v>
       </c>
       <c r="K10">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L10">
         <v>10</v>
@@ -77837,7 +77837,7 @@
         <v>9</v>
       </c>
       <c r="P10">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q10">
         <v>10</v>
@@ -77876,7 +77876,7 @@
         <v>-1</v>
       </c>
       <c r="AC10">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="AD10">
         <v>10</v>
@@ -77908,7 +77908,7 @@
         <v>124</v>
       </c>
       <c r="B11">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="C11">
         <v>7</v>
@@ -77935,7 +77935,7 @@
         <v>10</v>
       </c>
       <c r="K11">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L11">
         <v>7</v>
@@ -77950,7 +77950,7 @@
         <v>10</v>
       </c>
       <c r="P11">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q11">
         <v>10</v>
@@ -77989,7 +77989,7 @@
         <v>-1</v>
       </c>
       <c r="AC11">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="AD11">
         <v>7</v>
@@ -78021,7 +78021,7 @@
         <v>125</v>
       </c>
       <c r="B12">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="C12">
         <v>6</v>
@@ -78048,7 +78048,7 @@
         <v>10</v>
       </c>
       <c r="K12">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L12">
         <v>7</v>
@@ -78063,7 +78063,7 @@
         <v>9</v>
       </c>
       <c r="P12">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q12">
         <v>10</v>
@@ -78102,7 +78102,7 @@
         <v>-1</v>
       </c>
       <c r="AC12">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="AD12">
         <v>7</v>
@@ -78134,7 +78134,7 @@
         <v>126</v>
       </c>
       <c r="B13">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="C13">
         <v>6</v>
@@ -78161,7 +78161,7 @@
         <v>10</v>
       </c>
       <c r="K13">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L13">
         <v>8</v>
@@ -78176,7 +78176,7 @@
         <v>10</v>
       </c>
       <c r="P13">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q13">
         <v>10</v>
@@ -78215,7 +78215,7 @@
         <v>-1</v>
       </c>
       <c r="AC13">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="AD13">
         <v>7</v>
@@ -78247,7 +78247,7 @@
         <v>127</v>
       </c>
       <c r="B14">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="C14">
         <v>5</v>
@@ -78274,7 +78274,7 @@
         <v>10</v>
       </c>
       <c r="K14">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L14">
         <v>8</v>
@@ -78289,7 +78289,7 @@
         <v>9</v>
       </c>
       <c r="P14">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q14">
         <v>10</v>
@@ -78328,7 +78328,7 @@
         <v>-1</v>
       </c>
       <c r="AC14">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="AD14">
         <v>7</v>
@@ -78343,7 +78343,7 @@
         <v>9</v>
       </c>
       <c r="AH14">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AI14">
         <v>10</v>
@@ -78360,7 +78360,7 @@
         <v>128</v>
       </c>
       <c r="B15">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="C15">
         <v>7</v>
@@ -78387,7 +78387,7 @@
         <v>10</v>
       </c>
       <c r="K15">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L15">
         <v>8</v>
@@ -78402,7 +78402,7 @@
         <v>10</v>
       </c>
       <c r="P15">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q15">
         <v>10</v>
@@ -78441,7 +78441,7 @@
         <v>-1</v>
       </c>
       <c r="AC15">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="AD15">
         <v>8</v>
@@ -78473,7 +78473,7 @@
         <v>129</v>
       </c>
       <c r="B16">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="C16">
         <v>5</v>
@@ -78500,7 +78500,7 @@
         <v>5</v>
       </c>
       <c r="K16">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L16">
         <v>5</v>
@@ -78515,7 +78515,7 @@
         <v>5</v>
       </c>
       <c r="P16">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q16">
         <v>5</v>
@@ -78554,7 +78554,7 @@
         <v>-1</v>
       </c>
       <c r="AC16">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="AD16">
         <v>5</v>
@@ -78586,7 +78586,7 @@
         <v>130</v>
       </c>
       <c r="B17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="C17">
         <v>5</v>
@@ -78613,7 +78613,7 @@
         <v>5</v>
       </c>
       <c r="K17">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L17">
         <v>5</v>
@@ -78628,7 +78628,7 @@
         <v>8</v>
       </c>
       <c r="P17">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q17">
         <v>9</v>
@@ -78667,7 +78667,7 @@
         <v>-1</v>
       </c>
       <c r="AC17">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="AD17">
         <v>5</v>
@@ -78682,7 +78682,7 @@
         <v>8</v>
       </c>
       <c r="AH17">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AI17">
         <v>7</v>
@@ -78699,7 +78699,7 @@
         <v>131</v>
       </c>
       <c r="B18">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="C18">
         <v>6</v>
@@ -78726,7 +78726,7 @@
         <v>10</v>
       </c>
       <c r="K18">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L18">
         <v>9</v>
@@ -78741,7 +78741,7 @@
         <v>10</v>
       </c>
       <c r="P18">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q18">
         <v>10</v>
@@ -78780,7 +78780,7 @@
         <v>-1</v>
       </c>
       <c r="AC18">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="AD18">
         <v>8</v>
@@ -78812,7 +78812,7 @@
         <v>132</v>
       </c>
       <c r="B19">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="C19">
         <v>6</v>
@@ -78839,7 +78839,7 @@
         <v>10</v>
       </c>
       <c r="K19">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L19">
         <v>6</v>
@@ -78854,7 +78854,7 @@
         <v>9</v>
       </c>
       <c r="P19">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q19">
         <v>10</v>
@@ -78893,7 +78893,7 @@
         <v>-1</v>
       </c>
       <c r="AC19">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="AD19">
         <v>6</v>
@@ -78925,7 +78925,7 @@
         <v>133</v>
       </c>
       <c r="B20">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="C20">
         <v>5</v>
@@ -78952,7 +78952,7 @@
         <v>10</v>
       </c>
       <c r="K20">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L20">
         <v>7</v>
@@ -78967,7 +78967,7 @@
         <v>9</v>
       </c>
       <c r="P20">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q20">
         <v>10</v>
@@ -79006,7 +79006,7 @@
         <v>-1</v>
       </c>
       <c r="AC20">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="AD20">
         <v>6</v>
@@ -79038,7 +79038,7 @@
         <v>134</v>
       </c>
       <c r="B21">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="C21">
         <v>5</v>
@@ -79065,7 +79065,7 @@
         <v>5</v>
       </c>
       <c r="K21">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L21">
         <v>5</v>
@@ -79080,7 +79080,7 @@
         <v>5</v>
       </c>
       <c r="P21">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q21">
         <v>5</v>
@@ -79119,7 +79119,7 @@
         <v>-1</v>
       </c>
       <c r="AC21">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="AD21">
         <v>5</v>
@@ -79151,7 +79151,7 @@
         <v>135</v>
       </c>
       <c r="B22">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="C22">
         <v>6</v>
@@ -79178,7 +79178,7 @@
         <v>10</v>
       </c>
       <c r="K22">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L22">
         <v>7</v>
@@ -79193,7 +79193,7 @@
         <v>9</v>
       </c>
       <c r="P22">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q22">
         <v>10</v>
@@ -79232,7 +79232,7 @@
         <v>-1</v>
       </c>
       <c r="AC22">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="AD22">
         <v>7</v>
@@ -79264,7 +79264,7 @@
         <v>136</v>
       </c>
       <c r="B23">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="C23">
         <v>6</v>
@@ -79291,7 +79291,7 @@
         <v>10</v>
       </c>
       <c r="K23">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L23">
         <v>7</v>
@@ -79306,7 +79306,7 @@
         <v>9</v>
       </c>
       <c r="P23">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q23">
         <v>10</v>
@@ -79345,7 +79345,7 @@
         <v>-1</v>
       </c>
       <c r="AC23">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="AD23">
         <v>7</v>
@@ -79377,7 +79377,7 @@
         <v>137</v>
       </c>
       <c r="B24">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="C24">
         <v>8</v>
@@ -79404,7 +79404,7 @@
         <v>10</v>
       </c>
       <c r="K24">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L24">
         <v>9</v>
@@ -79419,7 +79419,7 @@
         <v>10</v>
       </c>
       <c r="P24">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q24">
         <v>10</v>
@@ -79458,7 +79458,7 @@
         <v>-1</v>
       </c>
       <c r="AC24">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AD24">
         <v>9</v>
@@ -79473,7 +79473,7 @@
         <v>10</v>
       </c>
       <c r="AH24">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AI24">
         <v>10</v>
@@ -79490,7 +79490,7 @@
         <v>138</v>
       </c>
       <c r="B25">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="C25">
         <v>5</v>
@@ -79517,7 +79517,7 @@
         <v>5</v>
       </c>
       <c r="K25">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L25">
         <v>5</v>
@@ -79532,7 +79532,7 @@
         <v>7</v>
       </c>
       <c r="P25">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q25">
         <v>8</v>
@@ -79571,7 +79571,7 @@
         <v>-1</v>
       </c>
       <c r="AC25">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="AD25">
         <v>5</v>
@@ -79586,7 +79586,7 @@
         <v>8</v>
       </c>
       <c r="AH25">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AI25">
         <v>8</v>
@@ -79603,7 +79603,7 @@
         <v>139</v>
       </c>
       <c r="B26">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="C26">
         <v>6</v>
@@ -79630,7 +79630,7 @@
         <v>10</v>
       </c>
       <c r="K26">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L26">
         <v>6</v>
@@ -79645,7 +79645,7 @@
         <v>9</v>
       </c>
       <c r="P26">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q26">
         <v>8</v>
@@ -79684,7 +79684,7 @@
         <v>-1</v>
       </c>
       <c r="AC26">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="AD26">
         <v>6</v>
@@ -79699,7 +79699,7 @@
         <v>9</v>
       </c>
       <c r="AH26">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AI26">
         <v>9</v>
@@ -79716,7 +79716,7 @@
         <v>140</v>
       </c>
       <c r="B27">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="C27">
         <v>5</v>
@@ -79743,7 +79743,7 @@
         <v>10</v>
       </c>
       <c r="K27">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L27">
         <v>5</v>
@@ -79758,7 +79758,7 @@
         <v>6</v>
       </c>
       <c r="P27">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q27">
         <v>8</v>
@@ -79797,7 +79797,7 @@
         <v>-1</v>
       </c>
       <c r="AC27">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="AD27">
         <v>5</v>
@@ -79829,7 +79829,7 @@
         <v>141</v>
       </c>
       <c r="B28">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="C28">
         <v>6</v>
@@ -79856,7 +79856,7 @@
         <v>10</v>
       </c>
       <c r="K28">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L28">
         <v>6</v>
@@ -79871,7 +79871,7 @@
         <v>9</v>
       </c>
       <c r="P28">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q28">
         <v>10</v>
@@ -79910,7 +79910,7 @@
         <v>-1</v>
       </c>
       <c r="AC28">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="AD28">
         <v>6</v>
@@ -79942,7 +79942,7 @@
         <v>142</v>
       </c>
       <c r="B29">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="C29">
         <v>5</v>
@@ -79969,7 +79969,7 @@
         <v>10</v>
       </c>
       <c r="K29">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L29">
         <v>7</v>
@@ -79984,7 +79984,7 @@
         <v>9</v>
       </c>
       <c r="P29">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q29">
         <v>10</v>
@@ -80023,7 +80023,7 @@
         <v>-1</v>
       </c>
       <c r="AC29">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="AD29">
         <v>6</v>
@@ -80055,7 +80055,7 @@
         <v>143</v>
       </c>
       <c r="B30">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="C30">
         <v>6</v>
@@ -80082,7 +80082,7 @@
         <v>10</v>
       </c>
       <c r="K30">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="L30">
         <v>10</v>
@@ -80097,7 +80097,7 @@
         <v>9</v>
       </c>
       <c r="P30">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q30">
         <v>10</v>
@@ -80136,7 +80136,7 @@
         <v>-1</v>
       </c>
       <c r="AC30">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AD30">
         <v>8</v>
@@ -80168,7 +80168,7 @@
         <v>144</v>
       </c>
       <c r="B31">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="C31">
         <v>8</v>
@@ -80195,7 +80195,7 @@
         <v>10</v>
       </c>
       <c r="K31">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L31">
         <v>8</v>
@@ -80210,7 +80210,7 @@
         <v>10</v>
       </c>
       <c r="P31">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q31">
         <v>10</v>
@@ -80249,7 +80249,7 @@
         <v>-1</v>
       </c>
       <c r="AC31">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="AD31">
         <v>8</v>
@@ -80281,7 +80281,7 @@
         <v>145</v>
       </c>
       <c r="B32">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="C32">
         <v>7</v>
@@ -80308,7 +80308,7 @@
         <v>10</v>
       </c>
       <c r="K32">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L32">
         <v>9</v>
@@ -80323,7 +80323,7 @@
         <v>10</v>
       </c>
       <c r="P32">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q32">
         <v>10</v>
@@ -80362,7 +80362,7 @@
         <v>-1</v>
       </c>
       <c r="AC32">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="AD32">
         <v>8</v>
@@ -80394,7 +80394,7 @@
         <v>146</v>
       </c>
       <c r="B33">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="C33">
         <v>8</v>
@@ -80421,7 +80421,7 @@
         <v>10</v>
       </c>
       <c r="K33">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L33">
         <v>10</v>
@@ -80436,7 +80436,7 @@
         <v>10</v>
       </c>
       <c r="P33">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q33">
         <v>10</v>
@@ -80475,7 +80475,7 @@
         <v>-1</v>
       </c>
       <c r="AC33">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="AD33">
         <v>9</v>
@@ -80507,7 +80507,7 @@
         <v>147</v>
       </c>
       <c r="B34">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="C34">
         <v>5</v>
@@ -80534,7 +80534,7 @@
         <v>10</v>
       </c>
       <c r="K34">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L34">
         <v>5</v>
@@ -80549,7 +80549,7 @@
         <v>8</v>
       </c>
       <c r="P34">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q34">
         <v>10</v>
@@ -80588,7 +80588,7 @@
         <v>-1</v>
       </c>
       <c r="AC34">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="AD34">
         <v>5</v>
@@ -80620,7 +80620,7 @@
         <v>148</v>
       </c>
       <c r="B35">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="C35">
         <v>5</v>
@@ -80647,7 +80647,7 @@
         <v>5</v>
       </c>
       <c r="K35">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L35">
         <v>5</v>
@@ -80662,7 +80662,7 @@
         <v>6</v>
       </c>
       <c r="P35">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q35">
         <v>7</v>
@@ -80701,7 +80701,7 @@
         <v>-1</v>
       </c>
       <c r="AC35">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="AD35">
         <v>5</v>
@@ -80716,7 +80716,7 @@
         <v>6</v>
       </c>
       <c r="AH35">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AI35">
         <v>6</v>
@@ -80733,7 +80733,7 @@
         <v>149</v>
       </c>
       <c r="B36">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="C36">
         <v>5</v>
@@ -80760,7 +80760,7 @@
         <v>5</v>
       </c>
       <c r="K36">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="L36">
         <v>5</v>
@@ -80775,7 +80775,7 @@
         <v>7</v>
       </c>
       <c r="P36">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q36">
         <v>5</v>
@@ -80814,7 +80814,7 @@
         <v>-1</v>
       </c>
       <c r="AC36">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="AD36">
         <v>5</v>
@@ -80829,7 +80829,7 @@
         <v>7</v>
       </c>
       <c r="AH36">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AI36">
         <v>5</v>
@@ -80846,7 +80846,7 @@
         <v>150</v>
       </c>
       <c r="B37">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="C37">
         <v>7</v>
@@ -80873,7 +80873,7 @@
         <v>10</v>
       </c>
       <c r="K37">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="L37">
         <v>9</v>
@@ -80888,7 +80888,7 @@
         <v>10</v>
       </c>
       <c r="P37">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q37">
         <v>10</v>
@@ -80927,7 +80927,7 @@
         <v>-1</v>
       </c>
       <c r="AC37">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AD37">
         <v>8</v>
@@ -80959,7 +80959,7 @@
         <v>151</v>
       </c>
       <c r="B38">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="C38">
         <v>10</v>
@@ -80986,7 +80986,7 @@
         <v>10</v>
       </c>
       <c r="K38">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L38">
         <v>10</v>
@@ -81001,7 +81001,7 @@
         <v>10</v>
       </c>
       <c r="P38">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q38">
         <v>10</v>
@@ -81040,7 +81040,7 @@
         <v>-1</v>
       </c>
       <c r="AC38">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="AD38">
         <v>10</v>
@@ -81295,7 +81295,7 @@
         <v>6</v>
       </c>
       <c r="O4">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P4">
         <v>7</v>
@@ -81307,7 +81307,7 @@
         <v>7</v>
       </c>
       <c r="S4">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T4">
         <v>-1</v>
@@ -81349,7 +81349,7 @@
         <v>7</v>
       </c>
       <c r="AG4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AH4">
         <v>6</v>
@@ -81408,7 +81408,7 @@
         <v>6</v>
       </c>
       <c r="O5">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P5">
         <v>5</v>
@@ -81420,7 +81420,7 @@
         <v>10</v>
       </c>
       <c r="S5">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T5">
         <v>-1</v>
@@ -81462,7 +81462,7 @@
         <v>8</v>
       </c>
       <c r="AG5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AH5">
         <v>7</v>
@@ -81521,7 +81521,7 @@
         <v>7</v>
       </c>
       <c r="O6">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P6">
         <v>5</v>
@@ -81533,7 +81533,7 @@
         <v>10</v>
       </c>
       <c r="S6">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T6">
         <v>-1</v>
@@ -81634,7 +81634,7 @@
         <v>7</v>
       </c>
       <c r="O7">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P7">
         <v>6</v>
@@ -81646,7 +81646,7 @@
         <v>6</v>
       </c>
       <c r="S7">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T7">
         <v>-1</v>
@@ -81688,7 +81688,7 @@
         <v>7</v>
       </c>
       <c r="AG7">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AH7">
         <v>5</v>
@@ -81747,7 +81747,7 @@
         <v>7</v>
       </c>
       <c r="O8">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="P8">
         <v>5</v>
@@ -81759,7 +81759,7 @@
         <v>9</v>
       </c>
       <c r="S8">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T8">
         <v>-1</v>
@@ -81801,7 +81801,7 @@
         <v>7</v>
       </c>
       <c r="AG8">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AH8">
         <v>7</v>
@@ -81860,7 +81860,7 @@
         <v>9</v>
       </c>
       <c r="O9">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P9">
         <v>8</v>
@@ -81872,7 +81872,7 @@
         <v>8</v>
       </c>
       <c r="S9">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T9">
         <v>-1</v>
@@ -81973,7 +81973,7 @@
         <v>9</v>
       </c>
       <c r="O10">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P10">
         <v>7</v>
@@ -81985,7 +81985,7 @@
         <v>7</v>
       </c>
       <c r="S10">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T10">
         <v>-1</v>
@@ -82027,7 +82027,7 @@
         <v>10</v>
       </c>
       <c r="AG10">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AH10">
         <v>6</v>
@@ -82086,7 +82086,7 @@
         <v>9</v>
       </c>
       <c r="O11">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="P11">
         <v>5</v>
@@ -82098,7 +82098,7 @@
         <v>7</v>
       </c>
       <c r="S11">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T11">
         <v>-1</v>
@@ -82199,7 +82199,7 @@
         <v>9</v>
       </c>
       <c r="O12">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P12">
         <v>10</v>
@@ -82211,7 +82211,7 @@
         <v>9</v>
       </c>
       <c r="S12">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T12">
         <v>-1</v>
@@ -82253,7 +82253,7 @@
         <v>10</v>
       </c>
       <c r="AG12">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AH12">
         <v>8</v>
@@ -82312,7 +82312,7 @@
         <v>9</v>
       </c>
       <c r="O13">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P13">
         <v>9</v>
@@ -82324,7 +82324,7 @@
         <v>8</v>
       </c>
       <c r="S13">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T13">
         <v>-1</v>
@@ -82366,7 +82366,7 @@
         <v>8</v>
       </c>
       <c r="AG13">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AH13">
         <v>8</v>
@@ -82425,7 +82425,7 @@
         <v>8</v>
       </c>
       <c r="O14">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P14">
         <v>9</v>
@@ -82437,7 +82437,7 @@
         <v>6</v>
       </c>
       <c r="S14">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T14">
         <v>-1</v>
@@ -82479,7 +82479,7 @@
         <v>8</v>
       </c>
       <c r="AG14">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AH14">
         <v>8</v>
@@ -82538,7 +82538,7 @@
         <v>5</v>
       </c>
       <c r="O15">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P15">
         <v>5</v>
@@ -82550,7 +82550,7 @@
         <v>5</v>
       </c>
       <c r="S15">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T15">
         <v>-1</v>
@@ -82592,7 +82592,7 @@
         <v>5</v>
       </c>
       <c r="AG15">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AH15">
         <v>5</v>
@@ -82651,7 +82651,7 @@
         <v>8</v>
       </c>
       <c r="O16">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="P16">
         <v>6</v>
@@ -82663,7 +82663,7 @@
         <v>8</v>
       </c>
       <c r="S16">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T16">
         <v>-1</v>
@@ -82764,7 +82764,7 @@
         <v>7</v>
       </c>
       <c r="O17">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P17">
         <v>10</v>
@@ -82776,7 +82776,7 @@
         <v>6</v>
       </c>
       <c r="S17">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T17">
         <v>-1</v>
@@ -82818,7 +82818,7 @@
         <v>7</v>
       </c>
       <c r="AG17">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AH17">
         <v>8</v>
@@ -82877,7 +82877,7 @@
         <v>9</v>
       </c>
       <c r="O18">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="P18">
         <v>5</v>
@@ -82889,7 +82889,7 @@
         <v>5</v>
       </c>
       <c r="S18">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T18">
         <v>-1</v>
@@ -82931,7 +82931,7 @@
         <v>9</v>
       </c>
       <c r="AG18">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AH18">
         <v>5</v>
@@ -82990,7 +82990,7 @@
         <v>9</v>
       </c>
       <c r="O19">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P19">
         <v>10</v>
@@ -83002,7 +83002,7 @@
         <v>7</v>
       </c>
       <c r="S19">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T19">
         <v>-1</v>
@@ -83103,7 +83103,7 @@
         <v>10</v>
       </c>
       <c r="O20">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P20">
         <v>10</v>
@@ -83115,7 +83115,7 @@
         <v>9</v>
       </c>
       <c r="S20">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T20">
         <v>-1</v>
@@ -83216,7 +83216,7 @@
         <v>10</v>
       </c>
       <c r="O21">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P21">
         <v>9</v>
@@ -83228,7 +83228,7 @@
         <v>10</v>
       </c>
       <c r="S21">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T21">
         <v>-1</v>
@@ -83329,7 +83329,7 @@
         <v>9</v>
       </c>
       <c r="O22">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="P22">
         <v>10</v>
@@ -83341,7 +83341,7 @@
         <v>6</v>
       </c>
       <c r="S22">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T22">
         <v>-1</v>
@@ -83442,7 +83442,7 @@
         <v>9</v>
       </c>
       <c r="O23">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="P23">
         <v>9</v>
@@ -83454,7 +83454,7 @@
         <v>9</v>
       </c>
       <c r="S23">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T23">
         <v>-1</v>
@@ -83496,7 +83496,7 @@
         <v>10</v>
       </c>
       <c r="AG23">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AH23">
         <v>9</v>
@@ -83555,7 +83555,7 @@
         <v>6</v>
       </c>
       <c r="O24">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P24">
         <v>5</v>
@@ -83567,7 +83567,7 @@
         <v>6</v>
       </c>
       <c r="S24">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T24">
         <v>-1</v>
@@ -83668,7 +83668,7 @@
         <v>10</v>
       </c>
       <c r="O25">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="P25">
         <v>10</v>
@@ -83680,7 +83680,7 @@
         <v>8</v>
       </c>
       <c r="S25">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T25">
         <v>-1</v>
@@ -83781,7 +83781,7 @@
         <v>8</v>
       </c>
       <c r="O26">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P26">
         <v>5</v>
@@ -83793,7 +83793,7 @@
         <v>7</v>
       </c>
       <c r="S26">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T26">
         <v>-1</v>
@@ -83835,7 +83835,7 @@
         <v>8</v>
       </c>
       <c r="AG26">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AH26">
         <v>6</v>
@@ -83894,7 +83894,7 @@
         <v>9</v>
       </c>
       <c r="O27">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P27">
         <v>5</v>
@@ -83906,7 +83906,7 @@
         <v>5</v>
       </c>
       <c r="S27">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T27">
         <v>-1</v>
@@ -84188,7 +84188,7 @@
         <v>6</v>
       </c>
       <c r="N4">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O4">
         <v>6</v>
@@ -84242,7 +84242,7 @@
         <v>8</v>
       </c>
       <c r="AF4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AG4">
         <v>8</v>
@@ -84301,7 +84301,7 @@
         <v>6</v>
       </c>
       <c r="N5">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O5">
         <v>5</v>
@@ -84355,7 +84355,7 @@
         <v>5</v>
       </c>
       <c r="AF5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AG5">
         <v>5</v>
@@ -84414,7 +84414,7 @@
         <v>10</v>
       </c>
       <c r="N6">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="O6">
         <v>10</v>
@@ -84527,7 +84527,7 @@
         <v>6</v>
       </c>
       <c r="N7">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O7">
         <v>7</v>
@@ -84581,7 +84581,7 @@
         <v>7</v>
       </c>
       <c r="AF7">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AG7">
         <v>8</v>
@@ -84640,7 +84640,7 @@
         <v>9</v>
       </c>
       <c r="N8">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O8">
         <v>8</v>
@@ -84753,7 +84753,7 @@
         <v>10</v>
       </c>
       <c r="N9">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O9">
         <v>10</v>
@@ -84866,7 +84866,7 @@
         <v>10</v>
       </c>
       <c r="N10">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="O10">
         <v>10</v>
@@ -84920,7 +84920,7 @@
         <v>10</v>
       </c>
       <c r="AF10">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AG10">
         <v>10</v>
@@ -84979,7 +84979,7 @@
         <v>10</v>
       </c>
       <c r="N11">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O11">
         <v>10</v>
@@ -85092,7 +85092,7 @@
         <v>5</v>
       </c>
       <c r="N12">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="O12">
         <v>8</v>
@@ -85205,7 +85205,7 @@
         <v>9</v>
       </c>
       <c r="N13">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O13">
         <v>10</v>
@@ -85259,7 +85259,7 @@
         <v>9</v>
       </c>
       <c r="AF13">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AG13">
         <v>10</v>
@@ -85318,7 +85318,7 @@
         <v>6</v>
       </c>
       <c r="N14">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="O14">
         <v>5</v>
@@ -85431,7 +85431,7 @@
         <v>9</v>
       </c>
       <c r="N15">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O15">
         <v>10</v>
@@ -85544,7 +85544,7 @@
         <v>6</v>
       </c>
       <c r="N16">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="O16">
         <v>9</v>
@@ -85657,7 +85657,7 @@
         <v>10</v>
       </c>
       <c r="N17">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="O17">
         <v>10</v>
@@ -85770,7 +85770,7 @@
         <v>10</v>
       </c>
       <c r="N18">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O18">
         <v>10</v>
@@ -85824,7 +85824,7 @@
         <v>10</v>
       </c>
       <c r="AF18">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AG18">
         <v>10</v>
@@ -85883,7 +85883,7 @@
         <v>10</v>
       </c>
       <c r="N19">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="O19">
         <v>10</v>
@@ -85937,7 +85937,7 @@
         <v>10</v>
       </c>
       <c r="AF19">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AG19">
         <v>10</v>
@@ -85996,7 +85996,7 @@
         <v>9</v>
       </c>
       <c r="N20">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O20">
         <v>9</v>
@@ -86050,7 +86050,7 @@
         <v>9</v>
       </c>
       <c r="AF20">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AG20">
         <v>10</v>
@@ -86109,7 +86109,7 @@
         <v>9</v>
       </c>
       <c r="N21">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O21">
         <v>10</v>
@@ -86163,7 +86163,7 @@
         <v>9</v>
       </c>
       <c r="AF21">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AG21">
         <v>10</v>
@@ -86222,7 +86222,7 @@
         <v>6</v>
       </c>
       <c r="N22">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O22">
         <v>9</v>
@@ -86276,7 +86276,7 @@
         <v>7</v>
       </c>
       <c r="AF22">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AG22">
         <v>9</v>
@@ -86335,7 +86335,7 @@
         <v>9</v>
       </c>
       <c r="N23">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O23">
         <v>10</v>
@@ -86389,7 +86389,7 @@
         <v>9</v>
       </c>
       <c r="AF23">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AG23">
         <v>10</v>
@@ -86448,7 +86448,7 @@
         <v>10</v>
       </c>
       <c r="N24">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="O24">
         <v>10</v>
@@ -86561,7 +86561,7 @@
         <v>10</v>
       </c>
       <c r="N25">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O25">
         <v>10</v>
@@ -86674,7 +86674,7 @@
         <v>10</v>
       </c>
       <c r="N26">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O26">
         <v>10</v>
@@ -86787,7 +86787,7 @@
         <v>7</v>
       </c>
       <c r="N27">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="O27">
         <v>9</v>
@@ -86841,7 +86841,7 @@
         <v>7</v>
       </c>
       <c r="AF27">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AG27">
         <v>9</v>
@@ -86900,7 +86900,7 @@
         <v>10</v>
       </c>
       <c r="N28">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="O28">
         <v>10</v>
@@ -87013,7 +87013,7 @@
         <v>9</v>
       </c>
       <c r="N29">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O29">
         <v>10</v>
@@ -87067,7 +87067,7 @@
         <v>9</v>
       </c>
       <c r="AF29">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AG29">
         <v>10</v>
@@ -87126,7 +87126,7 @@
         <v>10</v>
       </c>
       <c r="N30">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O30">
         <v>10</v>
@@ -87239,7 +87239,7 @@
         <v>6</v>
       </c>
       <c r="N31">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O31">
         <v>6</v>
@@ -87293,7 +87293,7 @@
         <v>7</v>
       </c>
       <c r="AF31">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AG31">
         <v>6</v>
@@ -87352,7 +87352,7 @@
         <v>6</v>
       </c>
       <c r="N32">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O32">
         <v>5</v>
@@ -87465,7 +87465,7 @@
         <v>9</v>
       </c>
       <c r="N33">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O33">
         <v>10</v>
@@ -87519,7 +87519,7 @@
         <v>9</v>
       </c>
       <c r="AF33">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AG33">
         <v>10</v>
@@ -87578,7 +87578,7 @@
         <v>7</v>
       </c>
       <c r="N34">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O34">
         <v>8</v>
@@ -87632,7 +87632,7 @@
         <v>8</v>
       </c>
       <c r="AF34">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AG34">
         <v>7</v>
@@ -87691,7 +87691,7 @@
         <v>6</v>
       </c>
       <c r="N35">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O35">
         <v>8</v>
@@ -87745,7 +87745,7 @@
         <v>6</v>
       </c>
       <c r="AF35">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AG35">
         <v>9</v>
@@ -87804,7 +87804,7 @@
         <v>7</v>
       </c>
       <c r="N36">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O36">
         <v>10</v>
@@ -87917,7 +87917,7 @@
         <v>9</v>
       </c>
       <c r="N37">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O37">
         <v>10</v>
@@ -88030,7 +88030,7 @@
         <v>6</v>
       </c>
       <c r="N38">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O38">
         <v>5</v>
@@ -88084,7 +88084,7 @@
         <v>7</v>
       </c>
       <c r="AF38">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AG38">
         <v>7</v>
@@ -88143,7 +88143,7 @@
         <v>8</v>
       </c>
       <c r="N39">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O39">
         <v>10</v>
@@ -88256,7 +88256,7 @@
         <v>10</v>
       </c>
       <c r="N40">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="O40">
         <v>10</v>
@@ -88310,7 +88310,7 @@
         <v>10</v>
       </c>
       <c r="AF40">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AG40">
         <v>10</v>
@@ -88369,7 +88369,7 @@
         <v>9</v>
       </c>
       <c r="N41">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O41">
         <v>10</v>
@@ -88423,7 +88423,7 @@
         <v>9</v>
       </c>
       <c r="AF41">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AG41">
         <v>10</v>

</xml_diff>

<commit_message>
Estadisticos Final ajustes materias
</commit_message>
<xml_diff>
--- a/Calificaciones20232.xlsx
+++ b/Calificaciones20232.xlsx
@@ -3780,7 +3780,7 @@
         <v>6</v>
       </c>
       <c r="AK4">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:37">
@@ -3893,7 +3893,7 @@
         <v>9</v>
       </c>
       <c r="AK5">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:37">
@@ -4006,7 +4006,7 @@
         <v>8</v>
       </c>
       <c r="AK6">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:37">
@@ -4119,7 +4119,7 @@
         <v>9</v>
       </c>
       <c r="AK7">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:37">
@@ -4232,7 +4232,7 @@
         <v>8</v>
       </c>
       <c r="AK8">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:37">
@@ -4345,7 +4345,7 @@
         <v>7</v>
       </c>
       <c r="AK9">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:37">
@@ -4458,7 +4458,7 @@
         <v>8</v>
       </c>
       <c r="AK10">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:37">
@@ -4571,7 +4571,7 @@
         <v>9</v>
       </c>
       <c r="AK11">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:37">
@@ -4684,7 +4684,7 @@
         <v>9</v>
       </c>
       <c r="AK12">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:37">
@@ -4797,7 +4797,7 @@
         <v>8</v>
       </c>
       <c r="AK13">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:37">
@@ -4910,7 +4910,7 @@
         <v>10</v>
       </c>
       <c r="AK14">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:37">
@@ -5023,7 +5023,7 @@
         <v>7</v>
       </c>
       <c r="AK15">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:37">
@@ -5136,7 +5136,7 @@
         <v>8</v>
       </c>
       <c r="AK16">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:37">
@@ -5249,7 +5249,7 @@
         <v>7</v>
       </c>
       <c r="AK17">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:37">
@@ -5362,7 +5362,7 @@
         <v>5</v>
       </c>
       <c r="AK18">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19" spans="1:37">
@@ -5475,7 +5475,7 @@
         <v>8</v>
       </c>
       <c r="AK19">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:37">
@@ -5588,7 +5588,7 @@
         <v>7</v>
       </c>
       <c r="AK20">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21" spans="1:37">
@@ -5701,7 +5701,7 @@
         <v>8</v>
       </c>
       <c r="AK21">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:37">
@@ -5814,7 +5814,7 @@
         <v>7</v>
       </c>
       <c r="AK22">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:37">
@@ -5927,7 +5927,7 @@
         <v>9</v>
       </c>
       <c r="AK23">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:37">
@@ -6040,7 +6040,7 @@
         <v>8</v>
       </c>
       <c r="AK24">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25" spans="1:37">
@@ -6153,7 +6153,7 @@
         <v>7</v>
       </c>
       <c r="AK25">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:37">
@@ -6266,7 +6266,7 @@
         <v>8</v>
       </c>
       <c r="AK26">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27" spans="1:37">
@@ -6379,7 +6379,7 @@
         <v>8</v>
       </c>
       <c r="AK27">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28" spans="1:37">
@@ -6492,7 +6492,7 @@
         <v>7</v>
       </c>
       <c r="AK28">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -32204,7 +32204,7 @@
         <v>8</v>
       </c>
       <c r="AK4">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:37">
@@ -32317,7 +32317,7 @@
         <v>7</v>
       </c>
       <c r="AK5">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:37">
@@ -32430,7 +32430,7 @@
         <v>9</v>
       </c>
       <c r="AK6">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:37">
@@ -32543,7 +32543,7 @@
         <v>9</v>
       </c>
       <c r="AK7">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:37">
@@ -32656,7 +32656,7 @@
         <v>5</v>
       </c>
       <c r="AK8">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:37">
@@ -32769,7 +32769,7 @@
         <v>7</v>
       </c>
       <c r="AK9">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:37">
@@ -32882,7 +32882,7 @@
         <v>9</v>
       </c>
       <c r="AK10">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:37">
@@ -32995,7 +32995,7 @@
         <v>5</v>
       </c>
       <c r="AK11">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:37">
@@ -33108,7 +33108,7 @@
         <v>7</v>
       </c>
       <c r="AK12">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:37">
@@ -33221,7 +33221,7 @@
         <v>7</v>
       </c>
       <c r="AK13">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:37">
@@ -33334,7 +33334,7 @@
         <v>6</v>
       </c>
       <c r="AK14">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:37">
@@ -33447,7 +33447,7 @@
         <v>7</v>
       </c>
       <c r="AK15">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:37">
@@ -33560,7 +33560,7 @@
         <v>6</v>
       </c>
       <c r="AK16">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:37">
@@ -33673,7 +33673,7 @@
         <v>8</v>
       </c>
       <c r="AK17">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:37">
@@ -33786,7 +33786,7 @@
         <v>6</v>
       </c>
       <c r="AK18">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19" spans="1:37">
@@ -33899,7 +33899,7 @@
         <v>8</v>
       </c>
       <c r="AK19">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:37">
@@ -34012,7 +34012,7 @@
         <v>7</v>
       </c>
       <c r="AK20">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21" spans="1:37">
@@ -34125,7 +34125,7 @@
         <v>7</v>
       </c>
       <c r="AK21">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:37">
@@ -34238,7 +34238,7 @@
         <v>5</v>
       </c>
       <c r="AK22">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23" spans="1:37">
@@ -34351,7 +34351,7 @@
         <v>10</v>
       </c>
       <c r="AK23">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:37">
@@ -34464,7 +34464,7 @@
         <v>7</v>
       </c>
       <c r="AK24">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25" spans="1:37">
@@ -34577,7 +34577,7 @@
         <v>8</v>
       </c>
       <c r="AK25">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:37">
@@ -34690,7 +34690,7 @@
         <v>8</v>
       </c>
       <c r="AK26">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27" spans="1:37">
@@ -34803,7 +34803,7 @@
         <v>8</v>
       </c>
       <c r="AK27">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28" spans="1:37">
@@ -34916,7 +34916,7 @@
         <v>6</v>
       </c>
       <c r="AK28">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="29" spans="1:37">
@@ -35029,7 +35029,7 @@
         <v>9</v>
       </c>
       <c r="AK29">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" spans="1:37">
@@ -35142,7 +35142,7 @@
         <v>5</v>
       </c>
       <c r="AK30">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31" spans="1:37">
@@ -35255,7 +35255,7 @@
         <v>8</v>
       </c>
       <c r="AK31">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="32" spans="1:37">
@@ -35368,7 +35368,7 @@
         <v>9</v>
       </c>
       <c r="AK32">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="33" spans="1:37">
@@ -35481,7 +35481,7 @@
         <v>5</v>
       </c>
       <c r="AK33">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -35775,7 +35775,7 @@
         <v>7</v>
       </c>
       <c r="AJ4">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK4">
         <v>8</v>
@@ -35888,7 +35888,7 @@
         <v>6</v>
       </c>
       <c r="AJ5">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK5">
         <v>7</v>
@@ -36001,7 +36001,7 @@
         <v>6</v>
       </c>
       <c r="AJ6">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK6">
         <v>6</v>
@@ -36114,7 +36114,7 @@
         <v>6</v>
       </c>
       <c r="AJ7">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK7">
         <v>7</v>
@@ -36227,7 +36227,7 @@
         <v>6</v>
       </c>
       <c r="AJ8">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK8">
         <v>6</v>
@@ -36340,7 +36340,7 @@
         <v>9</v>
       </c>
       <c r="AJ9">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK9">
         <v>8</v>
@@ -36453,7 +36453,7 @@
         <v>6</v>
       </c>
       <c r="AJ10">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK10">
         <v>8</v>
@@ -36566,7 +36566,7 @@
         <v>7</v>
       </c>
       <c r="AJ11">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK11">
         <v>8</v>
@@ -36679,7 +36679,7 @@
         <v>6</v>
       </c>
       <c r="AJ12">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK12">
         <v>8</v>
@@ -36792,7 +36792,7 @@
         <v>9</v>
       </c>
       <c r="AJ13">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK13">
         <v>9</v>
@@ -36905,7 +36905,7 @@
         <v>6</v>
       </c>
       <c r="AJ14">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK14">
         <v>7</v>
@@ -37018,7 +37018,7 @@
         <v>5</v>
       </c>
       <c r="AJ15">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="AK15">
         <v>5</v>
@@ -37131,7 +37131,7 @@
         <v>9</v>
       </c>
       <c r="AJ16">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK16">
         <v>8</v>
@@ -37244,7 +37244,7 @@
         <v>5</v>
       </c>
       <c r="AJ17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="AK17">
         <v>5</v>
@@ -37357,7 +37357,7 @@
         <v>5</v>
       </c>
       <c r="AJ18">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK18">
         <v>7</v>
@@ -37470,7 +37470,7 @@
         <v>6</v>
       </c>
       <c r="AJ19">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK19">
         <v>7</v>
@@ -37583,7 +37583,7 @@
         <v>6</v>
       </c>
       <c r="AJ20">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK20">
         <v>7</v>
@@ -37696,7 +37696,7 @@
         <v>5</v>
       </c>
       <c r="AJ21">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="AK21">
         <v>5</v>
@@ -37809,7 +37809,7 @@
         <v>7</v>
       </c>
       <c r="AJ22">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK22">
         <v>8</v>
@@ -37922,7 +37922,7 @@
         <v>5</v>
       </c>
       <c r="AJ23">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK23">
         <v>6</v>
@@ -38035,7 +38035,7 @@
         <v>7</v>
       </c>
       <c r="AJ24">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK24">
         <v>9</v>
@@ -38148,7 +38148,7 @@
         <v>8</v>
       </c>
       <c r="AJ25">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK25">
         <v>7</v>
@@ -38261,7 +38261,7 @@
         <v>8</v>
       </c>
       <c r="AJ26">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK26">
         <v>9</v>
@@ -38374,7 +38374,7 @@
         <v>5</v>
       </c>
       <c r="AJ27">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK27">
         <v>6</v>
@@ -38487,7 +38487,7 @@
         <v>7</v>
       </c>
       <c r="AJ28">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK28">
         <v>6</v>
@@ -38600,7 +38600,7 @@
         <v>7</v>
       </c>
       <c r="AJ29">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK29">
         <v>8</v>
@@ -38713,7 +38713,7 @@
         <v>8</v>
       </c>
       <c r="AJ30">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK30">
         <v>7</v>
@@ -38826,7 +38826,7 @@
         <v>9</v>
       </c>
       <c r="AJ31">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK31">
         <v>8</v>
@@ -38939,7 +38939,7 @@
         <v>5</v>
       </c>
       <c r="AJ32">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK32">
         <v>6</v>
@@ -39052,7 +39052,7 @@
         <v>6</v>
       </c>
       <c r="AJ33">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK33">
         <v>8</v>
@@ -39165,7 +39165,7 @@
         <v>9</v>
       </c>
       <c r="AJ34">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK34">
         <v>10</v>
@@ -39278,7 +39278,7 @@
         <v>7</v>
       </c>
       <c r="AJ35">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK35">
         <v>7</v>
@@ -39391,7 +39391,7 @@
         <v>9</v>
       </c>
       <c r="AJ36">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK36">
         <v>10</v>
@@ -39504,7 +39504,7 @@
         <v>7</v>
       </c>
       <c r="AJ37">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK37">
         <v>6</v>
@@ -39617,7 +39617,7 @@
         <v>8</v>
       </c>
       <c r="AJ38">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK38">
         <v>8</v>
@@ -39730,7 +39730,7 @@
         <v>6</v>
       </c>
       <c r="AJ39">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK39">
         <v>6</v>
@@ -39843,7 +39843,7 @@
         <v>5</v>
       </c>
       <c r="AJ40">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK40">
         <v>6</v>
@@ -39956,7 +39956,7 @@
         <v>8</v>
       </c>
       <c r="AJ41">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK41">
         <v>7</v>
@@ -40069,7 +40069,7 @@
         <v>6</v>
       </c>
       <c r="AJ42">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK42">
         <v>8</v>
@@ -40366,7 +40366,7 @@
         <v>6</v>
       </c>
       <c r="AJ4">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK4">
         <v>8</v>
@@ -40479,7 +40479,7 @@
         <v>5</v>
       </c>
       <c r="AJ5">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="AK5">
         <v>5</v>
@@ -40592,7 +40592,7 @@
         <v>5</v>
       </c>
       <c r="AJ6">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="AK6">
         <v>6</v>
@@ -40705,7 +40705,7 @@
         <v>6</v>
       </c>
       <c r="AJ7">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK7">
         <v>8</v>
@@ -40818,7 +40818,7 @@
         <v>6</v>
       </c>
       <c r="AJ8">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK8">
         <v>7</v>
@@ -40931,7 +40931,7 @@
         <v>6</v>
       </c>
       <c r="AJ9">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK9">
         <v>7</v>
@@ -41044,7 +41044,7 @@
         <v>7</v>
       </c>
       <c r="AJ10">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK10">
         <v>7</v>
@@ -41157,7 +41157,7 @@
         <v>7</v>
       </c>
       <c r="AJ11">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="AK11">
         <v>7</v>
@@ -41270,7 +41270,7 @@
         <v>6</v>
       </c>
       <c r="AJ12">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK12">
         <v>8</v>
@@ -41383,7 +41383,7 @@
         <v>6</v>
       </c>
       <c r="AJ13">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK13">
         <v>7</v>
@@ -41496,7 +41496,7 @@
         <v>5</v>
       </c>
       <c r="AJ14">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="AK14">
         <v>5</v>
@@ -41609,7 +41609,7 @@
         <v>5</v>
       </c>
       <c r="AJ15">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK15">
         <v>7</v>
@@ -41722,7 +41722,7 @@
         <v>5</v>
       </c>
       <c r="AJ16">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="AK16">
         <v>6</v>
@@ -41835,7 +41835,7 @@
         <v>5</v>
       </c>
       <c r="AJ17">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK17">
         <v>5</v>
@@ -41948,7 +41948,7 @@
         <v>5</v>
       </c>
       <c r="AJ18">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="AK18">
         <v>6</v>
@@ -42061,7 +42061,7 @@
         <v>5</v>
       </c>
       <c r="AJ19">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK19">
         <v>6</v>
@@ -42174,7 +42174,7 @@
         <v>5</v>
       </c>
       <c r="AJ20">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="AK20">
         <v>7</v>
@@ -42287,7 +42287,7 @@
         <v>5</v>
       </c>
       <c r="AJ21">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="AK21">
         <v>6</v>
@@ -42400,7 +42400,7 @@
         <v>6</v>
       </c>
       <c r="AJ22">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK22">
         <v>7</v>
@@ -42513,7 +42513,7 @@
         <v>6</v>
       </c>
       <c r="AJ23">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="AK23">
         <v>9</v>
@@ -42626,7 +42626,7 @@
         <v>5</v>
       </c>
       <c r="AJ24">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK24">
         <v>7</v>
@@ -42739,7 +42739,7 @@
         <v>5</v>
       </c>
       <c r="AJ25">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK25">
         <v>7</v>
@@ -42852,7 +42852,7 @@
         <v>6</v>
       </c>
       <c r="AJ26">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK26">
         <v>9</v>
@@ -42965,7 +42965,7 @@
         <v>6</v>
       </c>
       <c r="AJ27">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK27">
         <v>8</v>
@@ -43078,7 +43078,7 @@
         <v>5</v>
       </c>
       <c r="AJ28">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK28">
         <v>6</v>
@@ -43191,7 +43191,7 @@
         <v>5</v>
       </c>
       <c r="AJ29">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK29">
         <v>5</v>
@@ -43304,7 +43304,7 @@
         <v>6</v>
       </c>
       <c r="AJ30">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK30">
         <v>7</v>
@@ -43417,7 +43417,7 @@
         <v>5</v>
       </c>
       <c r="AJ31">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK31">
         <v>6</v>
@@ -43530,7 +43530,7 @@
         <v>5</v>
       </c>
       <c r="AJ32">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK32">
         <v>9</v>
@@ -43858,7 +43858,7 @@
         <v>6</v>
       </c>
       <c r="AO4">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:41">
@@ -43983,7 +43983,7 @@
         <v>6</v>
       </c>
       <c r="AO5">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:41">
@@ -44108,7 +44108,7 @@
         <v>5</v>
       </c>
       <c r="AO6">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:41">
@@ -44233,7 +44233,7 @@
         <v>5</v>
       </c>
       <c r="AO7">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:41">
@@ -44358,7 +44358,7 @@
         <v>6</v>
       </c>
       <c r="AO8">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:41">
@@ -44483,7 +44483,7 @@
         <v>5</v>
       </c>
       <c r="AO9">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:41">
@@ -44608,7 +44608,7 @@
         <v>5</v>
       </c>
       <c r="AO10">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:41">
@@ -44733,7 +44733,7 @@
         <v>6</v>
       </c>
       <c r="AO11">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:41">
@@ -44858,7 +44858,7 @@
         <v>6</v>
       </c>
       <c r="AO12">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:41">
@@ -44983,7 +44983,7 @@
         <v>5</v>
       </c>
       <c r="AO13">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:41">
@@ -45108,7 +45108,7 @@
         <v>5</v>
       </c>
       <c r="AO14">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:41">
@@ -45233,7 +45233,7 @@
         <v>5</v>
       </c>
       <c r="AO15">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:41">
@@ -45358,7 +45358,7 @@
         <v>6</v>
       </c>
       <c r="AO16">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:41">
@@ -45483,7 +45483,7 @@
         <v>5</v>
       </c>
       <c r="AO17">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:41">
@@ -45608,7 +45608,7 @@
         <v>6</v>
       </c>
       <c r="AO18">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:41">
@@ -45733,7 +45733,7 @@
         <v>6</v>
       </c>
       <c r="AO19">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:41">
@@ -45858,7 +45858,7 @@
         <v>6</v>
       </c>
       <c r="AO20">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21" spans="1:41">
@@ -45983,7 +45983,7 @@
         <v>6</v>
       </c>
       <c r="AO21">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:41">
@@ -46108,7 +46108,7 @@
         <v>6</v>
       </c>
       <c r="AO22">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:41">
@@ -46233,7 +46233,7 @@
         <v>7</v>
       </c>
       <c r="AO23">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:41">
@@ -46358,7 +46358,7 @@
         <v>6</v>
       </c>
       <c r="AO24">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25" spans="1:41">
@@ -46483,7 +46483,7 @@
         <v>6</v>
       </c>
       <c r="AO25">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:41">
@@ -46608,7 +46608,7 @@
         <v>5</v>
       </c>
       <c r="AO26">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -46905,7 +46905,7 @@
         <v>9</v>
       </c>
       <c r="AK4">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:37">
@@ -47018,7 +47018,7 @@
         <v>5</v>
       </c>
       <c r="AK5">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:37">
@@ -47131,7 +47131,7 @@
         <v>6</v>
       </c>
       <c r="AK6">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:37">
@@ -47244,7 +47244,7 @@
         <v>6</v>
       </c>
       <c r="AK7">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:37">
@@ -47357,7 +47357,7 @@
         <v>6</v>
       </c>
       <c r="AK8">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:37">
@@ -47470,7 +47470,7 @@
         <v>7</v>
       </c>
       <c r="AK9">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:37">
@@ -47583,7 +47583,7 @@
         <v>6</v>
       </c>
       <c r="AK10">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:37">
@@ -47696,7 +47696,7 @@
         <v>8</v>
       </c>
       <c r="AK11">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:37">
@@ -47809,7 +47809,7 @@
         <v>7</v>
       </c>
       <c r="AK12">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:37">
@@ -47922,7 +47922,7 @@
         <v>8</v>
       </c>
       <c r="AK13">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:37">
@@ -48035,7 +48035,7 @@
         <v>7</v>
       </c>
       <c r="AK14">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:37">
@@ -48148,7 +48148,7 @@
         <v>5</v>
       </c>
       <c r="AK15">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:37">
@@ -48261,7 +48261,7 @@
         <v>6</v>
       </c>
       <c r="AK16">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:37">
@@ -48374,7 +48374,7 @@
         <v>7</v>
       </c>
       <c r="AK17">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:37">
@@ -48487,7 +48487,7 @@
         <v>6</v>
       </c>
       <c r="AK18">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:37">
@@ -48600,7 +48600,7 @@
         <v>5</v>
       </c>
       <c r="AK19">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20" spans="1:37">
@@ -48713,7 +48713,7 @@
         <v>7</v>
       </c>
       <c r="AK20">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21" spans="1:37">
@@ -48826,7 +48826,7 @@
         <v>8</v>
       </c>
       <c r="AK21">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:37">
@@ -48939,7 +48939,7 @@
         <v>6</v>
       </c>
       <c r="AK22">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:37">
@@ -49052,7 +49052,7 @@
         <v>5</v>
       </c>
       <c r="AK23">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:37">
@@ -49165,7 +49165,7 @@
         <v>9</v>
       </c>
       <c r="AK24">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25" spans="1:37">
@@ -49278,7 +49278,7 @@
         <v>8</v>
       </c>
       <c r="AK25">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:37">
@@ -49420,7 +49420,7 @@
         <v>8</v>
       </c>
       <c r="AK27">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28" spans="1:37">
@@ -49533,7 +49533,7 @@
         <v>8</v>
       </c>
       <c r="AK28">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="29" spans="1:37">
@@ -49646,7 +49646,7 @@
         <v>7</v>
       </c>
       <c r="AK29">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" spans="1:37">
@@ -49759,7 +49759,7 @@
         <v>7</v>
       </c>
       <c r="AK30">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="31" spans="1:37">
@@ -49872,7 +49872,7 @@
         <v>8</v>
       </c>
       <c r="AK31">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="32" spans="1:37">
@@ -49985,7 +49985,7 @@
         <v>5</v>
       </c>
       <c r="AK32">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="33" spans="1:37">
@@ -50098,7 +50098,7 @@
         <v>5</v>
       </c>
       <c r="AK33">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="34" spans="1:37">
@@ -50211,7 +50211,7 @@
         <v>6</v>
       </c>
       <c r="AK34">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="35" spans="1:37">
@@ -50324,7 +50324,7 @@
         <v>6</v>
       </c>
       <c r="AK35">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="36" spans="1:37">
@@ -50437,7 +50437,7 @@
         <v>5</v>
       </c>
       <c r="AK36">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="37" spans="1:37">
@@ -50550,7 +50550,7 @@
         <v>6</v>
       </c>
       <c r="AK37">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -50847,7 +50847,7 @@
         <v>6</v>
       </c>
       <c r="AK4">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:37">
@@ -50960,7 +50960,7 @@
         <v>5</v>
       </c>
       <c r="AK5">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:37">
@@ -51073,7 +51073,7 @@
         <v>7</v>
       </c>
       <c r="AK6">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:37">
@@ -51186,7 +51186,7 @@
         <v>8</v>
       </c>
       <c r="AK7">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:37">
@@ -51299,7 +51299,7 @@
         <v>6</v>
       </c>
       <c r="AK8">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:37">
@@ -51412,7 +51412,7 @@
         <v>6</v>
       </c>
       <c r="AK9">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:37">
@@ -51525,7 +51525,7 @@
         <v>6</v>
       </c>
       <c r="AK10">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:37">
@@ -51638,7 +51638,7 @@
         <v>7</v>
       </c>
       <c r="AK11">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:37">
@@ -51751,7 +51751,7 @@
         <v>5</v>
       </c>
       <c r="AK12">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:37">
@@ -51864,7 +51864,7 @@
         <v>6</v>
       </c>
       <c r="AK13">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:37">
@@ -51977,7 +51977,7 @@
         <v>7</v>
       </c>
       <c r="AK14">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:37">
@@ -52090,7 +52090,7 @@
         <v>5</v>
       </c>
       <c r="AK15">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -66143,7 +66143,7 @@
         <v>6</v>
       </c>
       <c r="AO4">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:41">
@@ -66268,7 +66268,7 @@
         <v>9</v>
       </c>
       <c r="AO5">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:41">
@@ -66393,7 +66393,7 @@
         <v>7</v>
       </c>
       <c r="AO6">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:41">
@@ -66518,7 +66518,7 @@
         <v>6</v>
       </c>
       <c r="AO7">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:41">
@@ -66643,7 +66643,7 @@
         <v>6</v>
       </c>
       <c r="AO8">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:41">
@@ -66768,7 +66768,7 @@
         <v>6</v>
       </c>
       <c r="AO9">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:41">
@@ -66893,7 +66893,7 @@
         <v>6</v>
       </c>
       <c r="AO10">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:41">
@@ -67018,7 +67018,7 @@
         <v>6</v>
       </c>
       <c r="AO11">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:41">
@@ -67143,7 +67143,7 @@
         <v>7</v>
       </c>
       <c r="AO12">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:41">
@@ -67268,7 +67268,7 @@
         <v>7</v>
       </c>
       <c r="AO13">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:41">
@@ -67393,7 +67393,7 @@
         <v>8</v>
       </c>
       <c r="AO14">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:41">
@@ -67518,7 +67518,7 @@
         <v>6</v>
       </c>
       <c r="AO15">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:41">
@@ -67643,7 +67643,7 @@
         <v>8</v>
       </c>
       <c r="AO16">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:41">
@@ -67768,7 +67768,7 @@
         <v>5</v>
       </c>
       <c r="AO17">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:41">
@@ -67893,7 +67893,7 @@
         <v>8</v>
       </c>
       <c r="AO18">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:41">
@@ -68018,7 +68018,7 @@
         <v>6</v>
       </c>
       <c r="AO19">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:41">
@@ -68143,7 +68143,7 @@
         <v>7</v>
       </c>
       <c r="AO20">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21" spans="1:41">
@@ -68268,7 +68268,7 @@
         <v>6</v>
       </c>
       <c r="AO21">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:41">
@@ -68393,7 +68393,7 @@
         <v>6</v>
       </c>
       <c r="AO22">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:41">
@@ -68518,7 +68518,7 @@
         <v>7</v>
       </c>
       <c r="AO23">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:41">
@@ -68643,7 +68643,7 @@
         <v>8</v>
       </c>
       <c r="AO24">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25" spans="1:41">
@@ -68768,7 +68768,7 @@
         <v>5</v>
       </c>
       <c r="AO25">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:41">
@@ -68893,7 +68893,7 @@
         <v>7</v>
       </c>
       <c r="AO26">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27" spans="1:41">
@@ -69018,7 +69018,7 @@
         <v>9</v>
       </c>
       <c r="AO27">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28" spans="1:41">
@@ -69143,7 +69143,7 @@
         <v>6</v>
       </c>
       <c r="AO28">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="29" spans="1:41">
@@ -69268,7 +69268,7 @@
         <v>9</v>
       </c>
       <c r="AO29">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" spans="1:41">
@@ -69393,7 +69393,7 @@
         <v>10</v>
       </c>
       <c r="AO30">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="31" spans="1:41">
@@ -69518,7 +69518,7 @@
         <v>5</v>
       </c>
       <c r="AO31">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="32" spans="1:41">
@@ -69643,7 +69643,7 @@
         <v>6</v>
       </c>
       <c r="AO32">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="33" spans="1:41">
@@ -69768,7 +69768,7 @@
         <v>6</v>
       </c>
       <c r="AO33">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="34" spans="1:41">
@@ -69893,7 +69893,7 @@
         <v>6</v>
       </c>
       <c r="AO34">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -77462,7 +77462,7 @@
         <v>10</v>
       </c>
       <c r="AK4">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:37">
@@ -77575,7 +77575,7 @@
         <v>7</v>
       </c>
       <c r="AK5">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:37">
@@ -77688,7 +77688,7 @@
         <v>7</v>
       </c>
       <c r="AK6">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:37">
@@ -77801,7 +77801,7 @@
         <v>5</v>
       </c>
       <c r="AK7">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:37">
@@ -77914,7 +77914,7 @@
         <v>5</v>
       </c>
       <c r="AK8">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:37">
@@ -78027,7 +78027,7 @@
         <v>6</v>
       </c>
       <c r="AK9">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:37">
@@ -78140,7 +78140,7 @@
         <v>10</v>
       </c>
       <c r="AK10">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:37">
@@ -78253,7 +78253,7 @@
         <v>6</v>
       </c>
       <c r="AK11">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:37">
@@ -78366,7 +78366,7 @@
         <v>7</v>
       </c>
       <c r="AK12">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:37">
@@ -78479,7 +78479,7 @@
         <v>7</v>
       </c>
       <c r="AK13">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:37">
@@ -78592,7 +78592,7 @@
         <v>6</v>
       </c>
       <c r="AK14">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:37">
@@ -78705,7 +78705,7 @@
         <v>8</v>
       </c>
       <c r="AK15">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:37">
@@ -78818,7 +78818,7 @@
         <v>5</v>
       </c>
       <c r="AK16">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:37">
@@ -78931,7 +78931,7 @@
         <v>6</v>
       </c>
       <c r="AK17">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:37">
@@ -79044,7 +79044,7 @@
         <v>8</v>
       </c>
       <c r="AK18">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:37">
@@ -79157,7 +79157,7 @@
         <v>7</v>
       </c>
       <c r="AK19">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:37">
@@ -79270,7 +79270,7 @@
         <v>7</v>
       </c>
       <c r="AK20">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21" spans="1:37">
@@ -79383,7 +79383,7 @@
         <v>6</v>
       </c>
       <c r="AK21">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:37">
@@ -79496,7 +79496,7 @@
         <v>7</v>
       </c>
       <c r="AK22">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:37">
@@ -79609,7 +79609,7 @@
         <v>8</v>
       </c>
       <c r="AK23">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:37">
@@ -79722,7 +79722,7 @@
         <v>10</v>
       </c>
       <c r="AK24">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25" spans="1:37">
@@ -79835,7 +79835,7 @@
         <v>6</v>
       </c>
       <c r="AK25">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:37">
@@ -79948,7 +79948,7 @@
         <v>6</v>
       </c>
       <c r="AK26">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27" spans="1:37">
@@ -80061,7 +80061,7 @@
         <v>6</v>
       </c>
       <c r="AK27">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28" spans="1:37">
@@ -80174,7 +80174,7 @@
         <v>6</v>
       </c>
       <c r="AK28">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="29" spans="1:37">
@@ -80287,7 +80287,7 @@
         <v>6</v>
       </c>
       <c r="AK29">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" spans="1:37">
@@ -80400,7 +80400,7 @@
         <v>8</v>
       </c>
       <c r="AK30">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="31" spans="1:37">
@@ -80513,7 +80513,7 @@
         <v>7</v>
       </c>
       <c r="AK31">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="32" spans="1:37">
@@ -80626,7 +80626,7 @@
         <v>9</v>
       </c>
       <c r="AK32">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="33" spans="1:37">
@@ -80739,7 +80739,7 @@
         <v>8</v>
       </c>
       <c r="AK33">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="34" spans="1:37">
@@ -80852,7 +80852,7 @@
         <v>6</v>
       </c>
       <c r="AK34">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="35" spans="1:37">
@@ -80965,7 +80965,7 @@
         <v>5</v>
       </c>
       <c r="AK35">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="36" spans="1:37">
@@ -81078,7 +81078,7 @@
         <v>5</v>
       </c>
       <c r="AK36">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="37" spans="1:37">
@@ -81191,7 +81191,7 @@
         <v>8</v>
       </c>
       <c r="AK37">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="38" spans="1:37">
@@ -81304,7 +81304,7 @@
         <v>10</v>
       </c>
       <c r="AK38">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -81601,7 +81601,7 @@
         <v>6</v>
       </c>
       <c r="AK4">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:37">
@@ -81714,7 +81714,7 @@
         <v>9</v>
       </c>
       <c r="AK5">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:37">
@@ -81827,7 +81827,7 @@
         <v>9</v>
       </c>
       <c r="AK6">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:37">
@@ -81940,7 +81940,7 @@
         <v>6</v>
       </c>
       <c r="AK7">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:37">
@@ -82053,7 +82053,7 @@
         <v>8</v>
       </c>
       <c r="AK8">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:37">
@@ -82166,7 +82166,7 @@
         <v>9</v>
       </c>
       <c r="AK9">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:37">
@@ -82279,7 +82279,7 @@
         <v>8</v>
       </c>
       <c r="AK10">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:37">
@@ -82392,7 +82392,7 @@
         <v>8</v>
       </c>
       <c r="AK11">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:37">
@@ -82505,7 +82505,7 @@
         <v>9</v>
       </c>
       <c r="AK12">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:37">
@@ -82618,7 +82618,7 @@
         <v>8</v>
       </c>
       <c r="AK13">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:37">
@@ -82731,7 +82731,7 @@
         <v>7</v>
       </c>
       <c r="AK14">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:37">
@@ -82844,7 +82844,7 @@
         <v>6</v>
       </c>
       <c r="AK15">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:37">
@@ -82957,7 +82957,7 @@
         <v>8</v>
       </c>
       <c r="AK16">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:37">
@@ -83070,7 +83070,7 @@
         <v>6</v>
       </c>
       <c r="AK17">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:37">
@@ -83183,7 +83183,7 @@
         <v>7</v>
       </c>
       <c r="AK18">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:37">
@@ -83296,7 +83296,7 @@
         <v>8</v>
       </c>
       <c r="AK19">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:37">
@@ -83409,7 +83409,7 @@
         <v>9</v>
       </c>
       <c r="AK20">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21" spans="1:37">
@@ -83522,7 +83522,7 @@
         <v>9</v>
       </c>
       <c r="AK21">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:37">
@@ -83635,7 +83635,7 @@
         <v>8</v>
       </c>
       <c r="AK22">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:37">
@@ -83748,7 +83748,7 @@
         <v>9</v>
       </c>
       <c r="AK23">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:37">
@@ -83861,7 +83861,7 @@
         <v>6</v>
       </c>
       <c r="AK24">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25" spans="1:37">
@@ -83974,7 +83974,7 @@
         <v>9</v>
       </c>
       <c r="AK25">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:37">
@@ -84087,7 +84087,7 @@
         <v>8</v>
       </c>
       <c r="AK26">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27" spans="1:37">
@@ -84200,7 +84200,7 @@
         <v>6</v>
       </c>
       <c r="AK27">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -84494,7 +84494,7 @@
         <v>5</v>
       </c>
       <c r="AJ4">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK4">
         <v>6</v>
@@ -84607,7 +84607,7 @@
         <v>6</v>
       </c>
       <c r="AJ5">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK5">
         <v>6</v>
@@ -84720,7 +84720,7 @@
         <v>10</v>
       </c>
       <c r="AJ6">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK6">
         <v>10</v>
@@ -84833,7 +84833,7 @@
         <v>5</v>
       </c>
       <c r="AJ7">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK7">
         <v>8</v>
@@ -84946,7 +84946,7 @@
         <v>9</v>
       </c>
       <c r="AJ8">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK8">
         <v>8</v>
@@ -85059,7 +85059,7 @@
         <v>8</v>
       </c>
       <c r="AJ9">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK9">
         <v>9</v>
@@ -85172,7 +85172,7 @@
         <v>10</v>
       </c>
       <c r="AJ10">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK10">
         <v>9</v>
@@ -85285,7 +85285,7 @@
         <v>6</v>
       </c>
       <c r="AJ11">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK11">
         <v>9</v>
@@ -85398,7 +85398,7 @@
         <v>5</v>
       </c>
       <c r="AJ12">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK12">
         <v>7</v>
@@ -85511,7 +85511,7 @@
         <v>6</v>
       </c>
       <c r="AJ13">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK13">
         <v>8</v>
@@ -85624,7 +85624,7 @@
         <v>5</v>
       </c>
       <c r="AJ14">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="AK14">
         <v>5</v>
@@ -85737,7 +85737,7 @@
         <v>7</v>
       </c>
       <c r="AJ15">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK15">
         <v>9</v>
@@ -85850,7 +85850,7 @@
         <v>7</v>
       </c>
       <c r="AJ16">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK16">
         <v>9</v>
@@ -85963,7 +85963,7 @@
         <v>10</v>
       </c>
       <c r="AJ17">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK17">
         <v>10</v>
@@ -86076,7 +86076,7 @@
         <v>7</v>
       </c>
       <c r="AJ18">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK18">
         <v>9</v>
@@ -86189,7 +86189,7 @@
         <v>9</v>
       </c>
       <c r="AJ19">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK19">
         <v>8</v>
@@ -86302,7 +86302,7 @@
         <v>6</v>
       </c>
       <c r="AJ20">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK20">
         <v>8</v>
@@ -86415,7 +86415,7 @@
         <v>6</v>
       </c>
       <c r="AJ21">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK21">
         <v>7</v>
@@ -86528,7 +86528,7 @@
         <v>6</v>
       </c>
       <c r="AJ22">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK22">
         <v>8</v>
@@ -86641,7 +86641,7 @@
         <v>8</v>
       </c>
       <c r="AJ23">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK23">
         <v>9</v>
@@ -86754,7 +86754,7 @@
         <v>10</v>
       </c>
       <c r="AJ24">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK24">
         <v>10</v>
@@ -86867,7 +86867,7 @@
         <v>7</v>
       </c>
       <c r="AJ25">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK25">
         <v>8</v>
@@ -86980,7 +86980,7 @@
         <v>7</v>
       </c>
       <c r="AJ26">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK26">
         <v>9</v>
@@ -87093,7 +87093,7 @@
         <v>7</v>
       </c>
       <c r="AJ27">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK27">
         <v>6</v>
@@ -87206,7 +87206,7 @@
         <v>7</v>
       </c>
       <c r="AJ28">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK28">
         <v>7</v>
@@ -87319,7 +87319,7 @@
         <v>6</v>
       </c>
       <c r="AJ29">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK29">
         <v>7</v>
@@ -87432,7 +87432,7 @@
         <v>6</v>
       </c>
       <c r="AJ30">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK30">
         <v>6</v>
@@ -87545,7 +87545,7 @@
         <v>6</v>
       </c>
       <c r="AJ31">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK31">
         <v>8</v>
@@ -87658,7 +87658,7 @@
         <v>5</v>
       </c>
       <c r="AJ32">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK32">
         <v>6</v>
@@ -87771,7 +87771,7 @@
         <v>6</v>
       </c>
       <c r="AJ33">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK33">
         <v>7</v>
@@ -87884,7 +87884,7 @@
         <v>5</v>
       </c>
       <c r="AJ34">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK34">
         <v>6</v>
@@ -87997,7 +87997,7 @@
         <v>6</v>
       </c>
       <c r="AJ35">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK35">
         <v>7</v>
@@ -88110,7 +88110,7 @@
         <v>7</v>
       </c>
       <c r="AJ36">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK36">
         <v>8</v>
@@ -88223,7 +88223,7 @@
         <v>7</v>
       </c>
       <c r="AJ37">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK37">
         <v>8</v>
@@ -88336,7 +88336,7 @@
         <v>5</v>
       </c>
       <c r="AJ38">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK38">
         <v>6</v>
@@ -88449,7 +88449,7 @@
         <v>6</v>
       </c>
       <c r="AJ39">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK39">
         <v>9</v>
@@ -88562,7 +88562,7 @@
         <v>8</v>
       </c>
       <c r="AJ40">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK40">
         <v>9</v>
@@ -88675,7 +88675,7 @@
         <v>6</v>
       </c>
       <c r="AJ41">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AK41">
         <v>7</v>

</xml_diff>